<commit_message>
updated manuscript figures, analyses, and supplementary materials
</commit_message>
<xml_diff>
--- a/excel/PayGuard_Bayesian_Evaluation.xlsx
+++ b/excel/PayGuard_Bayesian_Evaluation.xlsx
@@ -663,7 +663,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>flydubai  |  PayGuard AI</t>
+          <t>PayGuard AI</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,19 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
+          <t>•  The interactive scorer uses 2,000 of the 4,000 saved posterior draws used for manuscript summaries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
           <t>•  This is the key advantage over the point-estimate regression: every prediction carries</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>•  its own uncertainty band, so borderline cases are visibly distinguished from confident ones.</t>
         </is>
@@ -773,7 +780,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>flydubai  |  PayGuard AI</t>
+          <t>PayGuard AI</t>
         </is>
       </c>
     </row>
@@ -69059,7 +69066,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>flydubai  |  PayGuard AI</t>
+          <t>PayGuard AI</t>
         </is>
       </c>
     </row>
@@ -69241,7 +69248,7 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Try setting bank_change = 1: the mean jumps toward ~100% and the interval stays tight (high confidence).</t>
+          <t>Vary the six displayed inputs to explore probabilities under the fitted approximate posterior.</t>
         </is>
       </c>
     </row>

</xml_diff>